<commit_message>
fix(plan): restore original Gantt grid and shift start date to 03/08/2026 to match Project baseline
</commit_message>
<xml_diff>
--- a/Ebooks/Plan_test.xlsx
+++ b/Ebooks/Plan_test.xlsx
@@ -615,7 +615,7 @@
   <sheetData>
     <row r="1" spans="6:80" x14ac:dyDescent="0.25">
       <c r="F1" s="2">
-        <v>46216</v>
+        <v>46237</v>
       </c>
       <c r="G1" s="2">
         <f>F1+1</f>
@@ -1524,7 +1524,7 @@
         <f>IF(C5&gt;0,INDEX(F$1:CB$1,MATCH("█",F5:CB5,0)),"")</f>
       </c>
       <c r="E5" s="11">
-        <f>IF(C5&gt;0,LOOKUP(2,1/(F5:CB5="█"),F$1:CB$1),"")</f>
+        <f>IF(C5&gt;0,INDEX(F$1:CB$1,MATCH("█",F5:CB5,0)+C5-1),"")</f>
       </c>
       <c r="F5" s="2" t="s">
         <v>27</v>
@@ -1618,7 +1618,7 @@
         <f>IF(C6&gt;0,INDEX(F$1:CB$1,MATCH("█",F6:CB6,0)),"")</f>
       </c>
       <c r="E6" s="11">
-        <f>IF(C6&gt;0,LOOKUP(2,1/(F6:CB6="█"),F$1:CB$1),"")</f>
+        <f>IF(C6&gt;0,INDEX(F$1:CB$1,MATCH("█",F6:CB6,0)+C6-1),"")</f>
       </c>
       <c r="F6" s="2" t="s">
         <v>27</v>
@@ -1712,7 +1712,7 @@
         <f>IF(C7&gt;0,INDEX(F$1:CB$1,MATCH("█",F7:CB7,0)),"")</f>
       </c>
       <c r="E7" s="11">
-        <f>IF(C7&gt;0,LOOKUP(2,1/(F7:CB7="█"),F$1:CB$1),"")</f>
+        <f>IF(C7&gt;0,INDEX(F$1:CB$1,MATCH("█",F7:CB7,0)+C7-1),"")</f>
       </c>
       <c r="F7" s="2" t="s">
         <v>27</v>
@@ -1806,7 +1806,7 @@
         <f>IF(C8&gt;0,INDEX(F$1:CB$1,MATCH("█",F8:CB8,0)),"")</f>
       </c>
       <c r="E8" s="11">
-        <f>IF(C8&gt;0,LOOKUP(2,1/(F8:CB8="█"),F$1:CB$1),"")</f>
+        <f>IF(C8&gt;0,INDEX(F$1:CB$1,MATCH("█",F8:CB8,0)+C8-1),"")</f>
       </c>
       <c r="F8" s="2" t="s">
         <v>27</v>
@@ -1900,7 +1900,7 @@
         <f>IF(C9&gt;0,INDEX(F$1:CB$1,MATCH("█",F9:CB9,0)),"")</f>
       </c>
       <c r="E9" s="11">
-        <f>IF(C9&gt;0,LOOKUP(2,1/(F9:CB9="█"),F$1:CB$1),"")</f>
+        <f>IF(C9&gt;0,INDEX(F$1:CB$1,MATCH("█",F9:CB9,0)+C9-1),"")</f>
       </c>
       <c r="F9" s="2" t="s">
         <v>27</v>
@@ -2236,7 +2236,7 @@
         <f>IF(C11&gt;0,INDEX(F$1:CB$1,MATCH("█",F11:CB11,0)),"")</f>
       </c>
       <c r="E11" s="11">
-        <f>IF(C11&gt;0,LOOKUP(2,1/(F11:CB11="█"),F$1:CB$1),"")</f>
+        <f>IF(C11&gt;0,INDEX(F$1:CB$1,MATCH("█",F11:CB11,0)+C11-1),"")</f>
       </c>
       <c r="F11" s="2" t="s">
         <v>27</v>
@@ -2330,7 +2330,7 @@
         <f>IF(C12&gt;0,INDEX(F$1:CB$1,MATCH("█",F12:CB12,0)),"")</f>
       </c>
       <c r="E12" s="11">
-        <f>IF(C12&gt;0,LOOKUP(2,1/(F12:CB12="█"),F$1:CB$1),"")</f>
+        <f>IF(C12&gt;0,INDEX(F$1:CB$1,MATCH("█",F12:CB12,0)+C12-1),"")</f>
       </c>
       <c r="F12" s="2" t="s">
         <v>27</v>
@@ -2424,7 +2424,7 @@
         <f>IF(C13&gt;0,INDEX(F$1:CB$1,MATCH("█",F13:CB13,0)),"")</f>
       </c>
       <c r="E13" s="11">
-        <f>IF(C13&gt;0,LOOKUP(2,1/(F13:CB13="█"),F$1:CB$1),"")</f>
+        <f>IF(C13&gt;0,INDEX(F$1:CB$1,MATCH("█",F13:CB13,0)+C13-1),"")</f>
       </c>
       <c r="F13" s="2" t="s">
         <v>27</v>
@@ -2518,7 +2518,7 @@
         <f>IF(C14&gt;0,INDEX(F$1:CB$1,MATCH("█",F14:CB14,0)),"")</f>
       </c>
       <c r="E14" s="11">
-        <f>IF(C14&gt;0,LOOKUP(2,1/(F14:CB14="█"),F$1:CB$1),"")</f>
+        <f>IF(C14&gt;0,INDEX(F$1:CB$1,MATCH("█",F14:CB14,0)+C14-1),"")</f>
       </c>
       <c r="F14" s="2" t="s">
         <v>27</v>
@@ -2854,7 +2854,7 @@
         <f>IF(C16&gt;0,INDEX(F$1:CB$1,MATCH("█",F16:CB16,0)),"")</f>
       </c>
       <c r="E16" s="11">
-        <f>IF(C16&gt;0,LOOKUP(2,1/(F16:CB16="█"),F$1:CB$1),"")</f>
+        <f>IF(C16&gt;0,INDEX(F$1:CB$1,MATCH("█",F16:CB16,0)+C16-1),"")</f>
       </c>
       <c r="F16" s="2" t="s">
         <v>27</v>
@@ -2948,7 +2948,7 @@
         <f>IF(C17&gt;0,INDEX(F$1:CB$1,MATCH("█",F17:CB17,0)),"")</f>
       </c>
       <c r="E17" s="11">
-        <f>IF(C17&gt;0,LOOKUP(2,1/(F17:CB17="█"),F$1:CB$1),"")</f>
+        <f>IF(C17&gt;0,INDEX(F$1:CB$1,MATCH("█",F17:CB17,0)+C17-1),"")</f>
       </c>
       <c r="F17" s="2" t="s">
         <v>27</v>
@@ -3042,7 +3042,7 @@
         <f>IF(C18&gt;0,INDEX(F$1:CB$1,MATCH("█",F18:CB18,0)),"")</f>
       </c>
       <c r="E18" s="11">
-        <f>IF(C18&gt;0,LOOKUP(2,1/(F18:CB18="█"),F$1:CB$1),"")</f>
+        <f>IF(C18&gt;0,INDEX(F$1:CB$1,MATCH("█",F18:CB18,0)+C18-1),"")</f>
       </c>
       <c r="F18" s="2" t="s">
         <v>27</v>
@@ -3136,7 +3136,7 @@
         <f>IF(C19&gt;0,INDEX(F$1:CB$1,MATCH("█",F19:CB19,0)),"")</f>
       </c>
       <c r="E19" s="11">
-        <f>IF(C19&gt;0,LOOKUP(2,1/(F19:CB19="█"),F$1:CB$1),"")</f>
+        <f>IF(C19&gt;0,INDEX(F$1:CB$1,MATCH("█",F19:CB19,0)+C19-1),"")</f>
       </c>
       <c r="F19" s="2" t="s">
         <v>27</v>
@@ -3230,7 +3230,7 @@
         <f>IF(C20&gt;0,INDEX(F$1:CB$1,MATCH("█",F20:CB20,0)),"")</f>
       </c>
       <c r="E20" s="11">
-        <f>IF(C20&gt;0,LOOKUP(2,1/(F20:CB20="█"),F$1:CB$1),"")</f>
+        <f>IF(C20&gt;0,INDEX(F$1:CB$1,MATCH("█",F20:CB20,0)+C20-1),"")</f>
       </c>
       <c r="F20" s="2" t="s">
         <v>27</v>
@@ -3324,7 +3324,7 @@
         <f>IF(C21&gt;0,INDEX(F$1:CB$1,MATCH("█",F21:CB21,0)),"")</f>
       </c>
       <c r="E21" s="11">
-        <f>IF(C21&gt;0,LOOKUP(2,1/(F21:CB21="█"),F$1:CB$1),"")</f>
+        <f>IF(C21&gt;0,INDEX(F$1:CB$1,MATCH("█",F21:CB21,0)+C21-1),"")</f>
       </c>
       <c r="F21" s="2" t="s">
         <v>27</v>
@@ -3418,7 +3418,7 @@
         <f>IF(C22&gt;0,INDEX(F$1:CB$1,MATCH("█",F22:CB22,0)),"")</f>
       </c>
       <c r="E22" s="11">
-        <f>IF(C22&gt;0,LOOKUP(2,1/(F22:CB22="█"),F$1:CB$1),"")</f>
+        <f>IF(C22&gt;0,INDEX(F$1:CB$1,MATCH("█",F22:CB22,0)+C22-1),"")</f>
       </c>
       <c r="F22" s="2" t="s">
         <v>27</v>
@@ -3512,7 +3512,7 @@
         <f>IF(C23&gt;0,INDEX(F$1:CB$1,MATCH("█",F23:CB23,0)),"")</f>
       </c>
       <c r="E23" s="11">
-        <f>IF(C23&gt;0,LOOKUP(2,1/(F23:CB23="█"),F$1:CB$1),"")</f>
+        <f>IF(C23&gt;0,INDEX(F$1:CB$1,MATCH("█",F23:CB23,0)+C23-1),"")</f>
       </c>
       <c r="F23" s="2" t="s">
         <v>27</v>
@@ -3606,7 +3606,7 @@
         <f>IF(C24&gt;0,INDEX(F$1:CB$1,MATCH("█",F24:CB24,0)),"")</f>
       </c>
       <c r="E24" s="11">
-        <f>IF(C24&gt;0,LOOKUP(2,1/(F24:CB24="█"),F$1:CB$1),"")</f>
+        <f>IF(C24&gt;0,INDEX(F$1:CB$1,MATCH("█",F24:CB24,0)+C24-1),"")</f>
       </c>
       <c r="F24" s="2" t="s">
         <v>27</v>
@@ -3700,7 +3700,7 @@
         <f>IF(C25&gt;0,INDEX(F$1:CB$1,MATCH("█",F25:CB25,0)),"")</f>
       </c>
       <c r="E25" s="11">
-        <f>IF(C25&gt;0,LOOKUP(2,1/(F25:CB25="█"),F$1:CB$1),"")</f>
+        <f>IF(C25&gt;0,INDEX(F$1:CB$1,MATCH("█",F25:CB25,0)+C25-1),"")</f>
       </c>
       <c r="F25" s="2" t="s">
         <v>27</v>

</xml_diff>